<commit_message>
progress: 13 village workbooks (sivaramans-llin 2026-10-08T19:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Manali_13.364448_80.04655.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Manali_13.364448_80.04655.xlsx
@@ -662,6 +662,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -669,6 +674,11 @@
           <t>117</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -676,6 +686,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -683,6 +698,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -690,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 3C, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -697,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -704,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -711,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -718,6 +758,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -725,6 +770,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -732,6 +782,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -739,6 +794,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -746,6 +806,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 4, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -753,6 +818,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -760,6 +830,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C1, 10C2, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -767,6 +842,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1B3, 1B4, 1B5, 1C1, 1C2, 1C3, 2A1, 2A2, 2B1, 2B2, 2C, 3, 4A1, 4A2, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -774,6 +854,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -781,6 +866,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -788,6 +878,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 3C, 3D, 4, 5, 6, 7A, 7B, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -795,6 +890,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 12A, 12B, 2, 3A, 3B, 4A, 4B, 4C, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -802,6 +902,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -809,6 +914,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -816,6 +926,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -823,6 +938,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -830,6 +950,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 5A, 5B, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -837,6 +962,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A1, 12A2, 12B, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -844,6 +974,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2, 3A1, 3A2, 3B1, 3B2, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -851,6 +986,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1A, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -858,6 +998,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -865,6 +1010,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -872,6 +1022,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -879,6 +1034,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -886,6 +1046,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -893,6 +1058,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -900,6 +1070,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -907,6 +1082,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -914,6 +1094,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 2A, 2B1, 2B2, 2C, 2D, 2E, 3A, 3B, 3C, 3D, 3E, 3F, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -921,6 +1106,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -928,6 +1118,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -935,6 +1130,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -942,6 +1142,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -949,6 +1154,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -956,6 +1166,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3A, 3B, 3C, 4A1A, 4A1B, 4A2, 4B, 5A1A, 5A1B, 5A2, 5B1, 5B2, 5B3, 5B4A, 5B4B, 5B5, 6, 7A, 7B, 7C, 7D, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -963,6 +1178,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>44A, 44B</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -970,6 +1190,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -977,6 +1202,11 @@
           <t>459</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -984,6 +1214,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -991,6 +1226,11 @@
           <t>460</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -998,6 +1238,11 @@
           <t>461</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1005,6 +1250,11 @@
           <t>462</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1012,6 +1262,11 @@
           <t>465</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1019,6 +1274,11 @@
           <t>466</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1026,6 +1286,11 @@
           <t>467</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1033,6 +1298,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1040,6 +1310,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1047,6 +1322,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1054,6 +1334,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1061,6 +1346,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1068,6 +1358,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15A, 15B, 16A, 16B1, 16B2, 17A, 17B, 17C, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1075,6 +1370,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1082,6 +1382,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 13C, 14, 15A, 15B, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1089,6 +1394,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1096,6 +1406,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1103,6 +1418,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11A, 11B, 11C, 11D, 11E, 11F, 11G, 11H1, 11H2, 11H3, 11I, 11J, 12A, 12B1, 12B2, 13, 14A, 14B, 14C, 14D, 15, 16, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C1A, 6C1B, 6C2, 6C3, 6C4, 6C5, 6C6, 7A, 7B, 8A, 8B, 8C, 8D, 8E, 9A1, 9A2, 9B1, 9B2, 9C1, 9C2, 9D1, 9D2, 9E1, 9E2, 9E3A, 9E3B1, 9E3B2</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1110,6 +1430,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1117,6 +1442,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1124,6 +1454,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1131,6 +1466,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1138,6 +1478,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2A4, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1145,6 +1490,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1152,6 +1502,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1159,6 +1514,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C, 2D, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1166,6 +1526,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1173,6 +1538,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1180,6 +1550,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1187,6 +1562,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1194,6 +1574,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1201,6 +1586,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1208,6 +1598,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1215,6 +1610,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1222,6 +1622,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1229,6 +1634,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1236,6 +1646,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1243,6 +1658,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2A, 2B2B</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1250,6 +1670,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1257,6 +1682,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1264,6 +1694,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1271,6 +1706,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1278,6 +1718,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1285,6 +1730,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B1, 1B2, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1292,6 +1742,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1299,6 +1754,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1306,6 +1766,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1313,6 +1778,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A1, 2A2, 2B1, 2B2, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1320,6 +1790,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 2</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1327,6 +1802,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1334,6 +1814,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A1, 11A2, 11B, 11C, 11D, 12A, 12B, 13A1, 13A2, 13B1, 13B2, 13C, 13D, 1A1, 1A2, 1B1, 1B2, 2A1, 2A2, 2B, 3A, 3B, 3C, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 4H, 5, 6A1, 6A10A, 6A10B, 6A11, 6A2, 6A3, 6A4, 6A5A1, 6A5A2, 6A5A3, 6A5B, 6A6A1, 6A6A2, 6A6A3, 6A6B, 6A7, 6A8A, 6A8B, 6A8C, 6A9, 6B, 6C, 6D1A, 6D1B, 6D2, 6D3A, 6D3B, 7A1, 7A2, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1341,6 +1826,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1348,6 +1838,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1355,6 +1850,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 2L, 3A1, 3A2, 3A3A, 3A3B, 3A3C, 3A4, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1362,6 +1862,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1369,11 +1874,21 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
           <t>91</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 16 village workbooks (sivaramans-llin 2026-10-08T19:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Manali_13.364448_80.04655.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Manali_13.364448_80.04655.xlsx
@@ -1898,6 +1898,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1, 1C2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1905,6 +1910,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1912,6 +1922,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1919,6 +1934,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4A, 4B, 4C, 4D, 4E, 4F, 5A, 5B, 6A, 6B, 6C, 6D, 6E, 7A, 7B, 8A1, 8A2, 8A3, 8A4, 8B1, 8B2, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1926,6 +1946,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1933,6 +1958,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1940,11 +1970,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>